<commit_message>
Changed calculation of MMS='grazing' to either 1) Based on grazing periods or 2) Based on dry matter intake (produces unreliable results)
</commit_message>
<xml_diff>
--- a/data/default/HorseHerd.xlsx
+++ b/data/default/HorseHerd.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="11400"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="8235"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="107">
   <si>
     <t>f_breed</t>
   </si>
@@ -324,6 +324,24 @@
   </si>
   <si>
     <t>HorseHerd-feed_rations.csv</t>
+  </si>
+  <si>
+    <t>Grazing</t>
+  </si>
+  <si>
+    <t>grazing_period</t>
+  </si>
+  <si>
+    <t>months</t>
+  </si>
+  <si>
+    <t>NIR 2022 page Table 5.9</t>
+  </si>
+  <si>
+    <t>indoors_during_grazing</t>
+  </si>
+  <si>
+    <t>Assumed included in the grazing period</t>
   </si>
 </sst>
 </file>
@@ -466,7 +484,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -548,8 +566,9 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
@@ -561,9 +580,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3290,7 +3309,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
@@ -3501,269 +3520,319 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:9" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E14" s="4"/>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:9" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+    </row>
+    <row r="16" spans="1:9" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E16" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="47">
+        <v>6</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="I16" s="41" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E17" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="F17" s="47">
+        <v>0</v>
+      </c>
+      <c r="G17" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="I17" s="41"/>
+    </row>
+    <row r="18" spans="1:9" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E18" s="4"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>3</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E20" t="s">
         <v>43</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F20" s="8">
         <v>0.5</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>6</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E21" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F21" s="8">
         <v>0.5</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>7</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E22" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F22" s="8">
         <f>0.5*1.05</f>
         <v>0.52500000000000002</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G22" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>8</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E23" t="s">
         <v>43</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F23" s="8">
         <f>0.5*1.1</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G23" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>3</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C24" t="s">
         <v>5</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E24" t="s">
         <v>43</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F24" s="8">
         <v>0.60721495776158751</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G24" t="s">
         <v>31</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H24" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>6</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C25" t="s">
         <v>5</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E25" t="s">
         <v>43</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F25" s="8">
         <v>0.60721495776158751</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G25" t="s">
         <v>31</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H25" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>7</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C26" t="s">
         <v>5</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E26" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F26" s="8">
         <v>0.63762671906630719</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G26" t="s">
         <v>31</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H26" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>8</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C27" t="s">
         <v>5</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E27" t="s">
         <v>43</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F27" s="8">
         <v>0.66878048717447958</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G27" t="s">
         <v>31</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H27" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E23" t="s">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E28" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F28" s="9">
         <f>( (0.15/2)*8 + 0.15 + 0.25 + 0.3 ) / 12</f>
         <v>0.10833333333333334</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H28" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E24" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E29" t="s">
         <v>26</v>
       </c>
-      <c r="F24" s="9">
+      <c r="F29" s="9">
         <f xml:space="preserve"> (1*3 + 0.7*1)/12</f>
         <v>0.30833333333333335</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H29" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C25" t="s">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
         <v>9</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E30" t="s">
         <v>24</v>
       </c>
-      <c r="F25">
+      <c r="F30">
         <v>0.25</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H30" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C26" t="s">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
         <v>10</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E31" t="s">
         <v>24</v>
       </c>
-      <c r="F26" s="9">
+      <c r="F31" s="9">
         <v>0.75</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H31" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C27" t="s">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
         <v>4</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E32" t="s">
         <v>24</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F32" s="9">
         <v>0.15</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H32" s="4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C28" t="s">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
         <v>5</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E33" t="s">
         <v>24</v>
       </c>
-      <c r="F28" s="28">
+      <c r="F33" s="28">
         <v>0</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H33" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5" t="s">
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E31" s="29" t="s">
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E36" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="F31" s="29">
+      <c r="F36" s="29">
         <v>0</v>
       </c>
-      <c r="G31" s="29"/>
-      <c r="H31" s="29" t="s">
+      <c r="G36" s="29"/>
+      <c r="H36" s="29" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E32" s="37" t="s">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E37" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F37" t="s">
         <v>100</v>
       </c>
     </row>
@@ -3839,10 +3908,10 @@
       <c r="N3" s="37" t="s">
         <v>85</v>
       </c>
-      <c r="O3" s="46" t="s">
+      <c r="O3" s="41" t="s">
         <v>97</v>
       </c>
-      <c r="P3" s="46" t="s">
+      <c r="P3" s="41" t="s">
         <v>98</v>
       </c>
       <c r="Q3" s="37" t="s">
@@ -3902,35 +3971,35 @@
         <v>32.999999999999993</v>
       </c>
       <c r="L4" s="9">
-        <f>$H4*L$25*100</f>
+        <f t="shared" ref="L4:S4" si="0">$H4*L$25*100</f>
         <v>0.23222788444440265</v>
       </c>
       <c r="M4" s="9">
-        <f>$H4*M$25*100</f>
+        <f t="shared" si="0"/>
         <v>2.39611841182896E-2</v>
       </c>
       <c r="N4" s="9">
-        <f>$H4*N$25*100</f>
+        <f t="shared" si="0"/>
         <v>8.3427301057299189E-2</v>
       </c>
       <c r="O4" s="9">
-        <f>$H4*O$25*100</f>
+        <f t="shared" si="0"/>
         <v>5.8354448396922961E-3</v>
       </c>
       <c r="P4" s="9">
-        <f>$H4*P$25*100</f>
+        <f t="shared" si="0"/>
         <v>0.14563835908849923</v>
       </c>
       <c r="Q4" s="9">
-        <f>$H4*Q$25*100</f>
+        <f t="shared" si="0"/>
         <v>6.5200501002148558E-4</v>
       </c>
       <c r="R4" s="9">
-        <f>$H4*R$25*100</f>
+        <f t="shared" si="0"/>
         <v>0.18662665404349996</v>
       </c>
       <c r="S4" s="9">
-        <f>$H4*S$25*100</f>
+        <f t="shared" si="0"/>
         <v>1.9931118668415414E-2</v>
       </c>
       <c r="T4" s="9">
@@ -3943,7 +4012,7 @@
       </c>
       <c r="V4" s="9"/>
       <c r="W4" s="9">
-        <f t="shared" ref="Q4:W19" si="0">$H4*W$25*100</f>
+        <f t="shared" ref="Q4:W19" si="1">$H4*W$25*100</f>
         <v>5.5308011194926036E-4</v>
       </c>
       <c r="X4" s="9">
@@ -3951,7 +4020,7 @@
         <v>9.5052213142011593E-2</v>
       </c>
       <c r="Z4" s="9">
-        <f>$H4*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" ref="Z4:Z19" si="2">$H4*SUM(Z$25,AA$25)*100</f>
         <v>3.7306677469965008E-2</v>
       </c>
       <c r="AB4" s="9"/>
@@ -3964,11 +4033,11 @@
         <v>10</v>
       </c>
       <c r="E5" s="36">
-        <f t="shared" ref="E5:E19" si="1">1-H5</f>
+        <f t="shared" ref="E5:E19" si="3">1-H5</f>
         <v>0.98</v>
       </c>
       <c r="F5" s="40">
-        <f t="shared" ref="F5:F19" si="2">1-G5</f>
+        <f t="shared" ref="F5:F19" si="4">1-G5</f>
         <v>0.83333333333333337</v>
       </c>
       <c r="G5" s="39">
@@ -3980,64 +4049,64 @@
       </c>
       <c r="I5" s="40"/>
       <c r="J5" s="38">
-        <f t="shared" ref="J5:J19" si="3">E5*F5*100</f>
+        <f t="shared" ref="J5:J19" si="5">E5*F5*100</f>
         <v>81.666666666666671</v>
       </c>
       <c r="K5" s="38">
-        <f t="shared" ref="K5:K19" si="4">E5*G5*100</f>
+        <f t="shared" ref="K5:K19" si="6">E5*G5*100</f>
         <v>16.333333333333332</v>
       </c>
       <c r="L5" s="9">
-        <f t="shared" ref="L5:L19" si="5">$H5*L$25*100</f>
+        <f t="shared" ref="L5:L19" si="7">$H5*L$25*100</f>
         <v>0.4644557688888053</v>
       </c>
       <c r="M5" s="9">
-        <f t="shared" ref="M4:N19" si="6">$H5*M$25*100</f>
+        <f t="shared" ref="M5:N19" si="8">$H5*M$25*100</f>
         <v>4.7922368236579201E-2</v>
       </c>
       <c r="N5" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.16685460211459838</v>
       </c>
       <c r="O5" s="9">
-        <f t="shared" ref="O4:P19" si="7">$H5*O$25*100</f>
+        <f t="shared" ref="O5:P19" si="9">$H5*O$25*100</f>
         <v>1.1670889679384592E-2</v>
       </c>
       <c r="P5" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.29127671817699846</v>
       </c>
       <c r="Q5" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.3040100200429712E-3</v>
       </c>
       <c r="R5" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.37325330808699991</v>
       </c>
       <c r="S5" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.9862237336830829E-2</v>
       </c>
       <c r="T5" s="9">
-        <f t="shared" ref="T5:T19" si="8">$H5*SUM(T$25,V$25*0.5)*100</f>
+        <f t="shared" ref="T5:T19" si="10">$H5*SUM(T$25,V$25*0.5)*100</f>
         <v>0.23473051574364462</v>
       </c>
       <c r="U5" s="9">
-        <f t="shared" ref="U5:U19" si="9">$H5*SUM(U$25,V$25*0.5)*100</f>
+        <f t="shared" ref="U5:U19" si="11">$H5*SUM(U$25,V$25*0.5)*100</f>
         <v>0.10284564026826409</v>
       </c>
       <c r="V5" s="9"/>
       <c r="W5" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.1061602238985207E-3</v>
       </c>
       <c r="X5" s="9">
-        <f t="shared" ref="X5:X19" si="10">$H5*SUM(X$25,Y$25)*100</f>
+        <f t="shared" ref="X5:X19" si="12">$H5*SUM(X$25,Y$25)*100</f>
         <v>0.19010442628402319</v>
       </c>
       <c r="Z5" s="9">
-        <f>$H5*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>7.4613354939930016E-2</v>
       </c>
       <c r="AB5" s="9"/>
@@ -4050,11 +4119,11 @@
         <v>4</v>
       </c>
       <c r="E6" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.92999999999999994</v>
       </c>
       <c r="F6" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.66666666666666674</v>
       </c>
       <c r="G6" s="39">
@@ -4066,64 +4135,64 @@
       </c>
       <c r="I6" s="40"/>
       <c r="J6" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>62</v>
       </c>
       <c r="K6" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>30.999999999999993</v>
       </c>
       <c r="L6" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.6255951911108186</v>
       </c>
       <c r="M6" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.16772828882802723</v>
       </c>
       <c r="N6" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.58399110740109439</v>
       </c>
       <c r="O6" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>4.0848113877846079E-2</v>
       </c>
       <c r="P6" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.0194685136194948</v>
       </c>
       <c r="Q6" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.5640350701503995E-3</v>
       </c>
       <c r="R6" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.3063865783044997</v>
       </c>
       <c r="S6" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.13951783067890791</v>
       </c>
       <c r="T6" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.82155680510275619</v>
       </c>
       <c r="U6" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.35995974093892436</v>
       </c>
       <c r="V6" s="9"/>
       <c r="W6" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.8715607836448231E-3</v>
       </c>
       <c r="X6" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.66536549199408124</v>
       </c>
       <c r="Z6" s="9">
-        <f>$H6*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.2611467422897551</v>
       </c>
       <c r="AB6" s="9"/>
@@ -4136,11 +4205,11 @@
         <v>5</v>
       </c>
       <c r="E7" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.92</v>
       </c>
       <c r="F7" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.66666666666666674</v>
       </c>
       <c r="G7" s="39">
@@ -4152,51 +4221,51 @@
       </c>
       <c r="I7" s="40"/>
       <c r="J7" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>61.333333333333343</v>
       </c>
       <c r="K7" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>30.666666666666664</v>
       </c>
       <c r="L7" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.8578230755552212</v>
       </c>
       <c r="M7" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.1916894729463168</v>
       </c>
       <c r="N7" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.66741840845839351</v>
       </c>
       <c r="O7" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>4.6683558717538369E-2</v>
       </c>
       <c r="P7" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.1651068727079938</v>
       </c>
       <c r="Q7" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.2160400801718847E-3</v>
       </c>
       <c r="R7" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.4930132323479997</v>
       </c>
       <c r="S7" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.15944894934732332</v>
       </c>
       <c r="T7" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.93892206297457848</v>
       </c>
       <c r="U7" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.41138256107305637</v>
       </c>
       <c r="V7" s="9"/>
@@ -4205,11 +4274,11 @@
         <v>4.4246408955940829E-3</v>
       </c>
       <c r="X7" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.76041770513609275</v>
       </c>
       <c r="Z7" s="9">
-        <f>$H7*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.29845341975972006</v>
       </c>
       <c r="AB7" s="9"/>
@@ -4222,7 +4291,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.99</v>
       </c>
       <c r="F8" s="40">
@@ -4238,56 +4307,56 @@
       </c>
       <c r="I8" s="40"/>
       <c r="J8" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>66</v>
       </c>
       <c r="K8" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>32.999999999999993</v>
       </c>
       <c r="L8" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.23222788444440265</v>
       </c>
       <c r="M8" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2.39611841182896E-2</v>
       </c>
       <c r="N8" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>8.3427301057299189E-2</v>
       </c>
       <c r="O8" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>5.8354448396922961E-3</v>
       </c>
       <c r="P8" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.14563835908849923</v>
       </c>
       <c r="Q8" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6.5200501002148558E-4</v>
       </c>
       <c r="R8" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.18662665404349996</v>
       </c>
       <c r="S8" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.9931118668415414E-2</v>
       </c>
       <c r="T8" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.11736525787182231</v>
       </c>
       <c r="U8" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>5.1422820134132047E-2</v>
       </c>
       <c r="V8" s="9"/>
       <c r="W8" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5308011194926036E-4</v>
       </c>
       <c r="X8" s="9">
@@ -4295,7 +4364,7 @@
         <v>9.5052213142011593E-2</v>
       </c>
       <c r="Z8" s="9">
-        <f>$H8*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>3.7306677469965008E-2</v>
       </c>
       <c r="AB8" s="9"/>
@@ -4308,11 +4377,11 @@
         <v>10</v>
       </c>
       <c r="E9" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.98</v>
       </c>
       <c r="F9" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.83333333333333337</v>
       </c>
       <c r="G9" s="39">
@@ -4324,64 +4393,64 @@
       </c>
       <c r="I9" s="40"/>
       <c r="J9" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>81.666666666666671</v>
       </c>
       <c r="K9" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>16.333333333333332</v>
       </c>
       <c r="L9" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.4644557688888053</v>
       </c>
       <c r="M9" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>4.7922368236579201E-2</v>
       </c>
       <c r="N9" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.16685460211459838</v>
       </c>
       <c r="O9" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.1670889679384592E-2</v>
       </c>
       <c r="P9" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.29127671817699846</v>
       </c>
       <c r="Q9" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.3040100200429712E-3</v>
       </c>
       <c r="R9" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.37325330808699991</v>
       </c>
       <c r="S9" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.9862237336830829E-2</v>
       </c>
       <c r="T9" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.23473051574364462</v>
       </c>
       <c r="U9" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.10284564026826409</v>
       </c>
       <c r="V9" s="9"/>
       <c r="W9" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.1061602238985207E-3</v>
       </c>
       <c r="X9" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.19010442628402319</v>
       </c>
       <c r="Z9" s="9">
-        <f>$H9*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>7.4613354939930016E-2</v>
       </c>
       <c r="AB9" s="9"/>
@@ -4394,11 +4463,11 @@
         <v>4</v>
       </c>
       <c r="E10" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.92999999999999994</v>
       </c>
       <c r="F10" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.66666666666666674</v>
       </c>
       <c r="G10" s="39">
@@ -4410,31 +4479,31 @@
       </c>
       <c r="I10" s="40"/>
       <c r="J10" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>62</v>
       </c>
       <c r="K10" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>30.999999999999993</v>
       </c>
       <c r="L10" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.6255951911108186</v>
       </c>
       <c r="M10" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.16772828882802723</v>
       </c>
       <c r="N10" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.58399110740109439</v>
       </c>
       <c r="O10" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>4.0848113877846079E-2</v>
       </c>
       <c r="P10" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.0194685136194948</v>
       </c>
       <c r="Q10" s="9">
@@ -4442,32 +4511,32 @@
         <v>4.5640350701503995E-3</v>
       </c>
       <c r="R10" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.3063865783044997</v>
       </c>
       <c r="S10" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.13951783067890791</v>
       </c>
       <c r="T10" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.82155680510275619</v>
       </c>
       <c r="U10" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.35995974093892436</v>
       </c>
       <c r="V10" s="9"/>
       <c r="W10" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.8715607836448231E-3</v>
       </c>
       <c r="X10" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.66536549199408124</v>
       </c>
       <c r="Z10" s="9">
-        <f>$H10*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.2611467422897551</v>
       </c>
       <c r="AB10" s="9"/>
@@ -4480,11 +4549,11 @@
         <v>5</v>
       </c>
       <c r="E11" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.97</v>
       </c>
       <c r="F11" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.66666666666666674</v>
       </c>
       <c r="G11" s="39">
@@ -4496,31 +4565,31 @@
       </c>
       <c r="I11" s="40"/>
       <c r="J11" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>64.666666666666671</v>
       </c>
       <c r="K11" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>32.333333333333329</v>
       </c>
       <c r="L11" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.69668365333320792</v>
       </c>
       <c r="M11" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>7.188355235486879E-2</v>
       </c>
       <c r="N11" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.25028190317189752</v>
       </c>
       <c r="O11" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.7506334519076888E-2</v>
       </c>
       <c r="P11" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.43691507726549772</v>
       </c>
       <c r="Q11" s="9">
@@ -4528,32 +4597,32 @@
         <v>1.9560150300644568E-3</v>
       </c>
       <c r="R11" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.55987996213049984</v>
       </c>
       <c r="S11" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.9793356005246247E-2</v>
       </c>
       <c r="T11" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.3520957736154669</v>
       </c>
       <c r="U11" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.15426846040239614</v>
       </c>
       <c r="V11" s="9"/>
       <c r="W11" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.659240335847781E-3</v>
       </c>
       <c r="X11" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.28515663942603475</v>
       </c>
       <c r="Z11" s="9">
-        <f>$H11*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.11192003240989502</v>
       </c>
       <c r="AB11" s="9"/>
@@ -4566,7 +4635,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.99</v>
       </c>
       <c r="F12" s="40">
@@ -4582,64 +4651,64 @@
       </c>
       <c r="I12" s="40"/>
       <c r="J12" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>66</v>
       </c>
       <c r="K12" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>32.999999999999993</v>
       </c>
       <c r="L12" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.23222788444440265</v>
       </c>
       <c r="M12" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2.39611841182896E-2</v>
       </c>
       <c r="N12" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>8.3427301057299189E-2</v>
       </c>
       <c r="O12" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>5.8354448396922961E-3</v>
       </c>
       <c r="P12" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.14563835908849923</v>
       </c>
       <c r="Q12" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6.5200501002148558E-4</v>
       </c>
       <c r="R12" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.18662665404349996</v>
       </c>
       <c r="S12" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.9931118668415414E-2</v>
       </c>
       <c r="T12" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.11736525787182231</v>
       </c>
       <c r="U12" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>5.1422820134132047E-2</v>
       </c>
       <c r="V12" s="9"/>
       <c r="W12" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5308011194926036E-4</v>
       </c>
       <c r="X12" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>9.5052213142011593E-2</v>
       </c>
       <c r="Z12" s="9">
-        <f>$H12*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>3.7306677469965008E-2</v>
       </c>
       <c r="AB12" s="9"/>
@@ -4652,11 +4721,11 @@
         <v>10</v>
       </c>
       <c r="E13" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.96</v>
       </c>
       <c r="F13" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.83333333333333337</v>
       </c>
       <c r="G13" s="39">
@@ -4668,64 +4737,64 @@
       </c>
       <c r="I13" s="40"/>
       <c r="J13" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>80</v>
       </c>
       <c r="K13" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>15.999999999999998</v>
       </c>
       <c r="L13" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.9289115377776106</v>
       </c>
       <c r="M13" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>9.5844736473158401E-2</v>
       </c>
       <c r="N13" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.33370920422919675</v>
       </c>
       <c r="O13" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.3341779358769184E-2</v>
       </c>
       <c r="P13" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.58255343635399692</v>
       </c>
       <c r="Q13" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.6080200400859423E-3</v>
       </c>
       <c r="R13" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.74650661617399983</v>
       </c>
       <c r="S13" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7.9724474673661658E-2</v>
       </c>
       <c r="T13" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.46946103148728924</v>
       </c>
       <c r="U13" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.20569128053652819</v>
       </c>
       <c r="V13" s="9"/>
       <c r="W13" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.2123204477970415E-3</v>
       </c>
       <c r="X13" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.38020885256804637</v>
       </c>
       <c r="Z13" s="9">
-        <f>$H13*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.14922670987986003</v>
       </c>
       <c r="AB13" s="9"/>
@@ -4738,11 +4807,11 @@
         <v>4</v>
       </c>
       <c r="E14" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.92999999999999994</v>
       </c>
       <c r="F14" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.66666666666666674</v>
       </c>
       <c r="G14" s="39">
@@ -4754,64 +4823,64 @@
       </c>
       <c r="I14" s="40"/>
       <c r="J14" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>62</v>
       </c>
       <c r="K14" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>30.999999999999993</v>
       </c>
       <c r="L14" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.6255951911108186</v>
       </c>
       <c r="M14" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.16772828882802723</v>
       </c>
       <c r="N14" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.58399110740109439</v>
       </c>
       <c r="O14" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>4.0848113877846079E-2</v>
       </c>
       <c r="P14" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.0194685136194948</v>
       </c>
       <c r="Q14" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.5640350701503995E-3</v>
       </c>
       <c r="R14" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.3063865783044997</v>
       </c>
       <c r="S14" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.13951783067890791</v>
       </c>
       <c r="T14" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.82155680510275619</v>
       </c>
       <c r="U14" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.35995974093892436</v>
       </c>
       <c r="V14" s="9"/>
       <c r="W14" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.8715607836448231E-3</v>
       </c>
       <c r="X14" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.66536549199408124</v>
       </c>
       <c r="Z14" s="9">
-        <f>$H14*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.2611467422897551</v>
       </c>
       <c r="AB14" s="9"/>
@@ -4824,11 +4893,11 @@
         <v>5</v>
       </c>
       <c r="E15" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.95</v>
       </c>
       <c r="F15" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.66666666666666674</v>
       </c>
       <c r="G15" s="39">
@@ -4840,64 +4909,64 @@
       </c>
       <c r="I15" s="40"/>
       <c r="J15" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>63.333333333333343</v>
       </c>
       <c r="K15" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>31.666666666666664</v>
       </c>
       <c r="L15" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.1611394222220133</v>
       </c>
       <c r="M15" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.11980592059144801</v>
       </c>
       <c r="N15" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.41713650528649598</v>
       </c>
       <c r="O15" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.9177224198461485E-2</v>
       </c>
       <c r="P15" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.72819179544249613</v>
       </c>
       <c r="Q15" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.2600250501074284E-3</v>
       </c>
       <c r="R15" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.93313327021749981</v>
       </c>
       <c r="S15" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9655593342077062E-2</v>
       </c>
       <c r="T15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.58682628935911163</v>
       </c>
       <c r="U15" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.25711410067066026</v>
       </c>
       <c r="V15" s="9"/>
       <c r="W15" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.7654005597463021E-3</v>
       </c>
       <c r="X15" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.47526106571005799</v>
       </c>
       <c r="Z15" s="9">
-        <f>$H15*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.18653338734982505</v>
       </c>
       <c r="AB15" s="9"/>
@@ -4910,7 +4979,7 @@
         <v>9</v>
       </c>
       <c r="E16" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.94</v>
       </c>
       <c r="F16" s="40">
@@ -4926,64 +4995,64 @@
       </c>
       <c r="I16" s="40"/>
       <c r="J16" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>62.666666666666671</v>
       </c>
       <c r="K16" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>31.333333333333329</v>
       </c>
       <c r="L16" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.3933673066664158</v>
       </c>
       <c r="M16" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.14376710470973758</v>
       </c>
       <c r="N16" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.50056380634379505</v>
       </c>
       <c r="O16" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>3.5012669038153775E-2</v>
       </c>
       <c r="P16" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.87383015453099544</v>
       </c>
       <c r="Q16" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.9120300601289135E-3</v>
       </c>
       <c r="R16" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.1197599242609997</v>
       </c>
       <c r="S16" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.11958671201049249</v>
       </c>
       <c r="T16" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.7041915472309338</v>
       </c>
       <c r="U16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.30853692080479228</v>
       </c>
       <c r="V16" s="9"/>
       <c r="W16" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3.318480671695562E-3</v>
       </c>
       <c r="X16" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.57031327885206951</v>
       </c>
       <c r="Z16" s="9">
-        <f>$H16*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.22384006481979005</v>
       </c>
       <c r="AB16" s="9"/>
@@ -4996,7 +5065,7 @@
         <v>10</v>
       </c>
       <c r="E17" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.89</v>
       </c>
       <c r="F17" s="40">
@@ -5024,52 +5093,52 @@
         <v>2.5545067288884291</v>
       </c>
       <c r="M17" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.26357302530118559</v>
       </c>
       <c r="N17" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.91770031163029109</v>
       </c>
       <c r="O17" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>6.4189893236615267E-2</v>
       </c>
       <c r="P17" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.6020219499734916</v>
       </c>
       <c r="Q17" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7.172055110236341E-3</v>
       </c>
       <c r="R17" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.0528931944784996</v>
       </c>
       <c r="S17" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.21924230535256958</v>
       </c>
       <c r="T17" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1.2910178365900453</v>
       </c>
       <c r="U17" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.56565102147545254</v>
       </c>
       <c r="V17" s="9"/>
       <c r="W17" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6.0838812314418641E-3</v>
       </c>
       <c r="X17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1.0455743445621275</v>
       </c>
       <c r="Z17" s="9">
-        <f>$H17*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.41037345216961513</v>
       </c>
       <c r="AB17" s="9"/>
@@ -5082,11 +5151,11 @@
         <v>4</v>
       </c>
       <c r="E18" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.9</v>
       </c>
       <c r="F18" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.66666666666666674</v>
       </c>
       <c r="G18" s="39">
@@ -5098,64 +5167,64 @@
       </c>
       <c r="I18" s="40"/>
       <c r="J18" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>60.000000000000007</v>
       </c>
       <c r="K18" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>30</v>
       </c>
       <c r="L18" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>2.3222788444440265</v>
       </c>
       <c r="M18" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.23961184118289602</v>
       </c>
       <c r="N18" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.83427301057299197</v>
       </c>
       <c r="O18" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>5.835444839692297E-2</v>
       </c>
       <c r="P18" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.4563835908849923</v>
       </c>
       <c r="Q18" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6.5200501002148567E-3</v>
       </c>
       <c r="R18" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.8662665404349996</v>
       </c>
       <c r="S18" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.19931118668415412</v>
       </c>
       <c r="T18" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1.1736525787182233</v>
       </c>
       <c r="U18" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.51422820134132052</v>
       </c>
       <c r="V18" s="9"/>
       <c r="W18" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.5308011194926043E-3</v>
       </c>
       <c r="X18" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>0.95052213142011599</v>
       </c>
       <c r="Z18" s="9">
-        <f>$H18*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.37306677469965011</v>
       </c>
       <c r="AB18" s="9"/>
@@ -5168,11 +5237,11 @@
         <v>5</v>
       </c>
       <c r="E19" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.88</v>
       </c>
       <c r="F19" s="40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.66666666666666674</v>
       </c>
       <c r="G19" s="39">
@@ -5184,64 +5253,64 @@
       </c>
       <c r="I19" s="40"/>
       <c r="J19" s="38">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>58.666666666666679</v>
       </c>
       <c r="K19" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>29.333333333333332</v>
       </c>
       <c r="L19" s="9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>2.7867346133328317</v>
       </c>
       <c r="M19" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.28753420941947516</v>
       </c>
       <c r="N19" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1.0011276126875901</v>
       </c>
       <c r="O19" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>7.002533807630755E-2</v>
       </c>
       <c r="P19" s="9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.7476603090619909</v>
       </c>
       <c r="Q19" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7.824060120257827E-3</v>
       </c>
       <c r="R19" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.2395198485219994</v>
       </c>
       <c r="S19" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.23917342402098499</v>
       </c>
       <c r="T19" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1.4083830944618676</v>
       </c>
       <c r="U19" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0.61707384160958456</v>
       </c>
       <c r="V19" s="9"/>
       <c r="W19" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6.6369613433911239E-3</v>
       </c>
       <c r="X19" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1.140626557704139</v>
       </c>
       <c r="Z19" s="9">
-        <f>$H19*SUM(Z$25,AA$25)*100</f>
+        <f t="shared" si="2"/>
         <v>0.44768012963958009</v>
       </c>
       <c r="AB19" s="9"/>
@@ -5264,10 +5333,10 @@
       <c r="N22" t="s">
         <v>67</v>
       </c>
-      <c r="O22" s="46" t="s">
+      <c r="O22" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="P22" s="46" t="s">
+      <c r="P22" s="41" t="s">
         <v>65</v>
       </c>
       <c r="Q22" t="s">
@@ -5285,7 +5354,7 @@
       <c r="U22" t="s">
         <v>70</v>
       </c>
-      <c r="V22" s="46" t="s">
+      <c r="V22" s="41" t="s">
         <v>95</v>
       </c>
       <c r="W22" t="s">
@@ -5294,13 +5363,13 @@
       <c r="X22" t="s">
         <v>72</v>
       </c>
-      <c r="Y22" s="46" t="s">
+      <c r="Y22" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="Z22" s="46" t="s">
+      <c r="Z22" s="41" t="s">
         <v>74</v>
       </c>
-      <c r="AA22" s="46" t="s">
+      <c r="AA22" s="41" t="s">
         <v>75</v>
       </c>
     </row>
@@ -5430,71 +5499,71 @@
         <v>79</v>
       </c>
       <c r="K25" s="35">
-        <f t="shared" ref="K25:AA25" si="11">SUM(K23:K24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="K25:L25" si="13">SUM(K23:K24)/SUM($K23:$K24)</f>
         <v>1</v>
       </c>
       <c r="L25" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0.23222788444440265</v>
       </c>
       <c r="M25" s="39">
-        <f t="shared" ref="M25" si="12">SUM(M23:M24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="M25" si="14">SUM(M23:M24)/SUM($K23:$K24)</f>
         <v>2.39611841182896E-2</v>
       </c>
       <c r="N25" s="39">
-        <f t="shared" ref="N25" si="13">SUM(N23:N24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="N25" si="15">SUM(N23:N24)/SUM($K23:$K24)</f>
         <v>8.3427301057299189E-2</v>
       </c>
       <c r="O25" s="39">
-        <f t="shared" ref="O25" si="14">SUM(O23:O24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="O25" si="16">SUM(O23:O24)/SUM($K23:$K24)</f>
         <v>5.8354448396922961E-3</v>
       </c>
       <c r="P25" s="39">
-        <f t="shared" ref="P25" si="15">SUM(P23:P24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="P25" si="17">SUM(P23:P24)/SUM($K23:$K24)</f>
         <v>0.14563835908849923</v>
       </c>
       <c r="Q25" s="39">
-        <f t="shared" ref="Q25" si="16">SUM(Q23:Q24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="Q25" si="18">SUM(Q23:Q24)/SUM($K23:$K24)</f>
         <v>6.5200501002148558E-4</v>
       </c>
       <c r="R25" s="39">
-        <f t="shared" ref="R25" si="17">SUM(R23:R24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="R25" si="19">SUM(R23:R24)/SUM($K23:$K24)</f>
         <v>0.18662665404349996</v>
       </c>
       <c r="S25" s="39">
-        <f t="shared" ref="S25" si="18">SUM(S23:S24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="S25" si="20">SUM(S23:S24)/SUM($K23:$K24)</f>
         <v>1.9931118668415414E-2</v>
       </c>
       <c r="T25" s="39">
-        <f t="shared" ref="T25" si="19">SUM(T23:T24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="T25" si="21">SUM(T23:T24)/SUM($K23:$K24)</f>
         <v>0.11183010068437482</v>
       </c>
       <c r="U25" s="39">
-        <f t="shared" ref="U25" si="20">SUM(U23:U24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="U25" si="22">SUM(U23:U24)/SUM($K23:$K24)</f>
         <v>4.588766294668456E-2</v>
       </c>
       <c r="V25" s="39">
-        <f t="shared" ref="V25" si="21">SUM(V23:V24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="V25" si="23">SUM(V23:V24)/SUM($K23:$K24)</f>
         <v>1.1070314374894972E-2</v>
       </c>
       <c r="W25" s="39">
-        <f t="shared" ref="W25" si="22">SUM(W23:W24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="W25" si="24">SUM(W23:W24)/SUM($K23:$K24)</f>
         <v>5.5308011194926036E-4</v>
       </c>
       <c r="X25" s="39">
-        <f t="shared" ref="X25" si="23">SUM(X23:X24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="X25" si="25">SUM(X23:X24)/SUM($K23:$K24)</f>
         <v>9.5052213142011593E-2</v>
       </c>
       <c r="Y25" s="39">
-        <f t="shared" ref="Y25" si="24">SUM(Y23:Y24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="Y25" si="26">SUM(Y23:Y24)/SUM($K23:$K24)</f>
         <v>0</v>
       </c>
       <c r="Z25" s="39">
-        <f t="shared" ref="Z25" si="25">SUM(Z23:Z24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="Z25" si="27">SUM(Z23:Z24)/SUM($K23:$K24)</f>
         <v>3.7306677469965008E-2</v>
       </c>
       <c r="AA25" s="39">
-        <f t="shared" ref="AA25" si="26">SUM(AA23:AA24)/SUM($K23:$K24)</f>
+        <f t="shared" ref="AA25" si="28">SUM(AA23:AA24)/SUM($K23:$K24)</f>
         <v>0</v>
       </c>
       <c r="AC25" s="40"/>
@@ -5524,55 +5593,55 @@
         <v>0</v>
       </c>
       <c r="O26" s="35">
-        <f t="shared" ref="O26:P26" si="27">O24/SUM(O23:O24)</f>
+        <f t="shared" ref="O26:P26" si="29">O24/SUM(O23:O24)</f>
         <v>0</v>
       </c>
       <c r="P26" s="35">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="Q26" s="35">
-        <f t="shared" ref="Q26:AA26" si="28">Q24/SUM(Q23:Q24)</f>
+        <f t="shared" ref="Q26:AA26" si="30">Q24/SUM(Q23:Q24)</f>
         <v>0</v>
       </c>
       <c r="R26" s="35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="S26" s="35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>0.243466817070878</v>
       </c>
       <c r="T26" s="35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>0.96019300361881776</v>
       </c>
       <c r="U26" s="35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="V26" s="35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="W26" s="35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>0.10975609756097561</v>
       </c>
       <c r="X26" s="35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="Y26" s="35" t="e">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
       <c r="Z26" s="35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="AA26" s="35" t="e">
-        <f t="shared" si="28"/>
+        <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -5852,25 +5921,25 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
-      <c r="M3" s="41"/>
-      <c r="N3" s="41"/>
-      <c r="O3" s="41"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="46"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="46"/>
     </row>
     <row r="4" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="43" t="s">
         <v>33</v>
       </c>
       <c r="C4" s="11"/>
@@ -5878,25 +5947,25 @@
         <v>34</v>
       </c>
       <c r="E4" s="11"/>
-      <c r="F4" s="44" t="s">
+      <c r="F4" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="44"/>
+      <c r="G4" s="45"/>
       <c r="H4" s="11"/>
-      <c r="I4" s="44" t="s">
+      <c r="I4" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="J4" s="44"/>
-      <c r="K4" s="44"/>
-      <c r="L4" s="44" t="s">
+      <c r="J4" s="45"/>
+      <c r="K4" s="45"/>
+      <c r="L4" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="M4" s="44"/>
-      <c r="N4" s="44"/>
+      <c r="M4" s="45"/>
+      <c r="N4" s="45"/>
       <c r="O4" s="13"/>
     </row>
     <row r="5" spans="2:21" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B5" s="43"/>
+      <c r="B5" s="44"/>
       <c r="C5" s="14" t="s">
         <v>38</v>
       </c>
@@ -6544,41 +6613,41 @@
       </c>
     </row>
     <row r="17" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B17" s="45" t="s">
+      <c r="B17" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="45"/>
-      <c r="H17" s="45"/>
-      <c r="I17" s="45"/>
-      <c r="J17" s="45"/>
-      <c r="K17" s="45"/>
-      <c r="L17" s="45"/>
-      <c r="M17" s="45"/>
-      <c r="N17" s="45"/>
-      <c r="O17" s="45"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="42"/>
+      <c r="J17" s="42"/>
+      <c r="K17" s="42"/>
+      <c r="L17" s="42"/>
+      <c r="M17" s="42"/>
+      <c r="N17" s="42"/>
+      <c r="O17" s="42"/>
     </row>
     <row r="18" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B18" s="45"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="45"/>
-      <c r="J18" s="45"/>
-      <c r="K18" s="45"/>
-      <c r="L18" s="45"/>
-      <c r="M18" s="45"/>
-      <c r="N18" s="45"/>
-      <c r="O18" s="45"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="42"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="42"/>
+      <c r="L18" s="42"/>
+      <c r="M18" s="42"/>
+      <c r="N18" s="42"/>
+      <c r="O18" s="42"/>
     </row>
     <row r="19" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B19" s="42" t="s">
+      <c r="B19" s="43" t="s">
         <v>33</v>
       </c>
       <c r="C19" s="11"/>
@@ -6586,25 +6655,25 @@
         <v>34</v>
       </c>
       <c r="E19" s="11"/>
-      <c r="F19" s="44" t="s">
+      <c r="F19" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="G19" s="44"/>
+      <c r="G19" s="45"/>
       <c r="H19" s="11"/>
-      <c r="I19" s="44" t="s">
+      <c r="I19" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="J19" s="44"/>
-      <c r="K19" s="44"/>
-      <c r="L19" s="44" t="s">
+      <c r="J19" s="45"/>
+      <c r="K19" s="45"/>
+      <c r="L19" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="M19" s="44"/>
-      <c r="N19" s="44"/>
+      <c r="M19" s="45"/>
+      <c r="N19" s="45"/>
       <c r="O19" s="13"/>
     </row>
     <row r="20" spans="2:21" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B20" s="43"/>
+      <c r="B20" s="44"/>
       <c r="C20" s="14" t="s">
         <v>38</v>
       </c>
@@ -7253,16 +7322,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B3:O3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="L4:N4"/>
     <mergeCell ref="B17:O18"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="I19:K19"/>
     <mergeCell ref="L19:N19"/>
-    <mergeCell ref="B3:O3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="L4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>